<commit_message>
Atualização da tabela de requisitos funcionais, não funcionais e regra de negócios
</commit_message>
<xml_diff>
--- a/Cronograma(2ºSemestre).xlsx
+++ b/Cronograma(2ºSemestre).xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DTG-2026\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DTG-2026\Desktop\Patinhas Felizes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{45A9D593-8C9E-4AE1-9B68-937FFA1CD28C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2F3D9DD-F6C8-48DB-8A90-0DF62698F83B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{08C7B1D9-FAF1-4333-ABBB-F5A2186B84FB}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>ATIVIDADES</t>
   </si>
@@ -105,6 +105,12 @@
   </si>
   <si>
     <t>Definição do objetivo do website</t>
+  </si>
+  <si>
+    <t>Mínimo:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Máximo: </t>
   </si>
 </sst>
 </file>
@@ -167,11 +173,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -189,6 +192,16 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -523,7 +536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3F214DF-C21D-4A8B-8694-9ACBEE2BE205}">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="45.5546875" customWidth="1"/>
@@ -534,333 +547,351 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="4">
-        <v>46239</v>
-      </c>
-      <c r="C3" s="5">
-        <v>1</v>
-      </c>
-      <c r="D3" s="4">
-        <v>46239</v>
-      </c>
-      <c r="E3" s="6">
-        <v>1</v>
-      </c>
-      <c r="F3" s="6">
+      <c r="B3" s="3">
+        <v>46239</v>
+      </c>
+      <c r="C3" s="4">
+        <v>1</v>
+      </c>
+      <c r="D3" s="3">
+        <v>46239</v>
+      </c>
+      <c r="E3" s="5">
+        <v>1</v>
+      </c>
+      <c r="F3" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="4">
-        <v>46239</v>
-      </c>
-      <c r="C4" s="5">
-        <v>1</v>
-      </c>
-      <c r="D4" s="4">
-        <v>46239</v>
-      </c>
-      <c r="E4" s="6">
-        <v>1</v>
-      </c>
-      <c r="F4" s="6">
+      <c r="B4" s="3">
+        <v>46239</v>
+      </c>
+      <c r="C4" s="4">
+        <v>1</v>
+      </c>
+      <c r="D4" s="3">
+        <v>46239</v>
+      </c>
+      <c r="E4" s="5">
+        <v>1</v>
+      </c>
+      <c r="F4" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="4">
-        <v>46239</v>
-      </c>
-      <c r="C5" s="5">
-        <v>1</v>
-      </c>
-      <c r="D5" s="4">
-        <v>46239</v>
-      </c>
-      <c r="E5" s="6">
-        <v>1</v>
-      </c>
-      <c r="F5" s="6">
+      <c r="B5" s="3">
+        <v>46239</v>
+      </c>
+      <c r="C5" s="4">
+        <v>1</v>
+      </c>
+      <c r="D5" s="3">
+        <v>46239</v>
+      </c>
+      <c r="E5" s="5">
+        <v>1</v>
+      </c>
+      <c r="F5" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="4">
-        <v>46239</v>
-      </c>
-      <c r="C6" s="5">
-        <v>1</v>
-      </c>
-      <c r="D6" s="4">
-        <v>46239</v>
-      </c>
-      <c r="E6" s="6">
-        <v>1</v>
-      </c>
-      <c r="F6" s="6">
+      <c r="B6" s="3">
+        <v>46239</v>
+      </c>
+      <c r="C6" s="4">
+        <v>1</v>
+      </c>
+      <c r="D6" s="3">
+        <v>46239</v>
+      </c>
+      <c r="E6" s="5">
+        <v>1</v>
+      </c>
+      <c r="F6" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="7">
         <v>46244</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="4">
         <v>2</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="7">
         <v>46246</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="5">
         <v>0</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="8">
-        <v>46239</v>
-      </c>
-      <c r="C8" s="5">
-        <v>1</v>
-      </c>
-      <c r="D8" s="8">
-        <v>46239</v>
-      </c>
-      <c r="E8" s="6">
-        <v>1</v>
-      </c>
-      <c r="F8" s="6">
+      <c r="B8" s="7">
+        <v>46239</v>
+      </c>
+      <c r="C8" s="4">
+        <v>1</v>
+      </c>
+      <c r="D8" s="7">
+        <v>46239</v>
+      </c>
+      <c r="E8" s="5">
+        <v>1</v>
+      </c>
+      <c r="F8" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="8">
-        <v>46239</v>
-      </c>
-      <c r="C9" s="5">
-        <v>1</v>
-      </c>
-      <c r="D9" s="8">
-        <v>46239</v>
-      </c>
-      <c r="E9" s="6">
-        <v>1</v>
-      </c>
-      <c r="F9" s="6">
+      <c r="B9" s="7">
+        <v>46239</v>
+      </c>
+      <c r="C9" s="4">
+        <v>1</v>
+      </c>
+      <c r="D9" s="7">
+        <v>46239</v>
+      </c>
+      <c r="E9" s="5">
+        <v>1</v>
+      </c>
+      <c r="F9" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10" s="7">
         <v>46244</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="4">
         <v>2</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="7">
         <v>46246</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="5">
         <v>0</v>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="8">
+      <c r="B11" s="7">
         <v>46251</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="4">
         <v>29</v>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="7">
         <v>46281</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="5">
         <v>0</v>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="7">
         <v>46251</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12" s="4">
         <v>29</v>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="7">
+        <v>46351</v>
+      </c>
+      <c r="E12" s="5">
+        <v>0</v>
+      </c>
+      <c r="F12" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" s="7">
+        <v>46251</v>
+      </c>
+      <c r="C13" s="4">
+        <v>29</v>
+      </c>
+      <c r="D13" s="7">
         <v>46281</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E13" s="5">
         <v>0</v>
       </c>
-      <c r="F12" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13" s="8">
-        <v>46251</v>
-      </c>
-      <c r="C13" s="5">
-        <v>29</v>
-      </c>
-      <c r="D13" s="8">
-        <v>46281</v>
-      </c>
-      <c r="E13" s="6">
+      <c r="F13" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" s="7">
+        <v>46286</v>
+      </c>
+      <c r="C14" s="4">
+        <v>35</v>
+      </c>
+      <c r="D14" s="7">
+        <v>46321</v>
+      </c>
+      <c r="E14" s="5">
         <v>0</v>
       </c>
-      <c r="F13" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B14" s="8">
+      <c r="F14" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" s="7">
         <v>46286</v>
       </c>
-      <c r="C14" s="5">
+      <c r="C15" s="4">
         <v>35</v>
       </c>
-      <c r="D14" s="8">
+      <c r="D15" s="7">
         <v>46321</v>
       </c>
-      <c r="E14" s="6">
+      <c r="E15" s="5">
         <v>0</v>
       </c>
-      <c r="F14" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B15" s="8">
-        <v>46286</v>
-      </c>
-      <c r="C15" s="5">
-        <v>35</v>
-      </c>
-      <c r="D15" s="8">
-        <v>46321</v>
-      </c>
-      <c r="E15" s="6">
+      <c r="F15" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" s="7">
+        <v>46323</v>
+      </c>
+      <c r="C16" s="4">
+        <v>36</v>
+      </c>
+      <c r="D16" s="7">
+        <v>46358</v>
+      </c>
+      <c r="E16" s="5">
         <v>0</v>
       </c>
-      <c r="F15" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B16" s="8">
+      <c r="F16" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" s="7">
         <v>46323</v>
       </c>
-      <c r="C16" s="5">
+      <c r="C17" s="4">
         <v>36</v>
       </c>
-      <c r="D16" s="8">
+      <c r="D17" s="7">
         <v>46358</v>
       </c>
-      <c r="E16" s="6">
+      <c r="E17" s="5">
         <v>0</v>
       </c>
-      <c r="F16" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B17" s="8">
-        <v>46323</v>
-      </c>
-      <c r="C17" s="5">
-        <v>36</v>
-      </c>
-      <c r="D17" s="8">
+      <c r="F17" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="10">
+        <f>MIN(D3:D17)</f>
+        <v>46239</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" s="10">
+        <f>MAX(D3:D17)</f>
         <v>46358</v>
-      </c>
-      <c r="E17" s="6">
-        <v>0</v>
-      </c>
-      <c r="F17" s="6">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>